<commit_message>
improve handling of specialization
</commit_message>
<xml_diff>
--- a/CCS COURSE LIST.xlsx
+++ b/CCS COURSE LIST.xlsx
@@ -1,14 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Downloads\LOGOS\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="0" windowWidth="2370" windowHeight="0"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="First Semester" sheetId="1" r:id="rId4"/>
-    <sheet state="visible" name="Second Semester" sheetId="2" r:id="rId5"/>
-    <sheet state="visible" name="Midyear" sheetId="3" r:id="rId6"/>
+    <sheet name="First Semester" sheetId="1" r:id="rId1"/>
+    <sheet name="Second Semester" sheetId="2" r:id="rId2"/>
+    <sheet name="Midyear" sheetId="3" r:id="rId3"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -732,24 +740,26 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="4">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
     <font>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
     <font>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
@@ -759,62 +769,55 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="8">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="right" readingOrder="0" vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -1004,21 +1007,24 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:F107"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="17.88"/>
-    <col customWidth="1" min="2" max="2" width="66.0"/>
+    <col min="1" max="1" width="17.85546875" customWidth="1"/>
+    <col min="2" max="2" width="66" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1038,7 +1044,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -1049,16 +1055,16 @@
         <v>8</v>
       </c>
       <c r="D2" s="3">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E2" s="3">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F2" s="3">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>9</v>
       </c>
@@ -1069,16 +1075,16 @@
         <v>8</v>
       </c>
       <c r="D3" s="3">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E3" s="3">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F3" s="3">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>11</v>
       </c>
@@ -1089,16 +1095,16 @@
         <v>8</v>
       </c>
       <c r="D4" s="3">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E4" s="3">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F4" s="3">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>13</v>
       </c>
@@ -1109,16 +1115,16 @@
         <v>8</v>
       </c>
       <c r="D5" s="3">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E5" s="3">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F5" s="3">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>15</v>
       </c>
@@ -1129,16 +1135,16 @@
         <v>8</v>
       </c>
       <c r="D6" s="3">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E6" s="3">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F6" s="3">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>17</v>
       </c>
@@ -1149,16 +1155,16 @@
         <v>8</v>
       </c>
       <c r="D7" s="3">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E7" s="3">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F7" s="3">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>19</v>
       </c>
@@ -1169,16 +1175,16 @@
         <v>8</v>
       </c>
       <c r="D8" s="3">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E8" s="3">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F8" s="3">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>21</v>
       </c>
@@ -1189,16 +1195,16 @@
         <v>8</v>
       </c>
       <c r="D9" s="3">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E9" s="3">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F9" s="3">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>23</v>
       </c>
@@ -1209,16 +1215,16 @@
         <v>8</v>
       </c>
       <c r="D10" s="3">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E10" s="3">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F10" s="3">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>25</v>
       </c>
@@ -1229,16 +1235,16 @@
         <v>8</v>
       </c>
       <c r="D11" s="3">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E11" s="3">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F11" s="3">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="12">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>27</v>
       </c>
@@ -1249,16 +1255,16 @@
         <v>8</v>
       </c>
       <c r="D12" s="3">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E12" s="3">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F12" s="3">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="13">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>29</v>
       </c>
@@ -1269,16 +1275,16 @@
         <v>8</v>
       </c>
       <c r="D13" s="3">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E13" s="3">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F13" s="3">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="14">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>31</v>
       </c>
@@ -1289,16 +1295,16 @@
         <v>8</v>
       </c>
       <c r="D14" s="3">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E14" s="3">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F14" s="3">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>33</v>
       </c>
@@ -1309,16 +1315,16 @@
         <v>8</v>
       </c>
       <c r="D15" s="3">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E15" s="3">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F15" s="3">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="16">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>35</v>
       </c>
@@ -1329,16 +1335,16 @@
         <v>8</v>
       </c>
       <c r="D16" s="3">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E16" s="3">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F16" s="3">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="17">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>37</v>
       </c>
@@ -1349,16 +1355,16 @@
         <v>8</v>
       </c>
       <c r="D17" s="3">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E17" s="3">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F17" s="3">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="18">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>39</v>
       </c>
@@ -1369,16 +1375,16 @@
         <v>8</v>
       </c>
       <c r="D18" s="3">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E18" s="3">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F18" s="3">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="19">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>41</v>
       </c>
@@ -1389,16 +1395,16 @@
         <v>8</v>
       </c>
       <c r="D19" s="3">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E19" s="3">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F19" s="3">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="20">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>43</v>
       </c>
@@ -1409,16 +1415,16 @@
         <v>8</v>
       </c>
       <c r="D20" s="3">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E20" s="3">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F20" s="3">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="21">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>45</v>
       </c>
@@ -1429,16 +1435,16 @@
         <v>8</v>
       </c>
       <c r="D21" s="3">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E21" s="3">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F21" s="3">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="22">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>47</v>
       </c>
@@ -1449,16 +1455,16 @@
         <v>8</v>
       </c>
       <c r="D22" s="3">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E22" s="3">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F22" s="3">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="23">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>49</v>
       </c>
@@ -1469,16 +1475,16 @@
         <v>8</v>
       </c>
       <c r="D23" s="3">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E23" s="3">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F23" s="3">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="24">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>51</v>
       </c>
@@ -1489,16 +1495,16 @@
         <v>8</v>
       </c>
       <c r="D24" s="3">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E24" s="3">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F24" s="3">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>53</v>
       </c>
@@ -1509,16 +1515,16 @@
         <v>8</v>
       </c>
       <c r="D25" s="3">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E25" s="3">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F25" s="3">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="26">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>55</v>
       </c>
@@ -1529,16 +1535,16 @@
         <v>8</v>
       </c>
       <c r="D26" s="3">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="E26" s="3">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="F26" s="3">
-        <v>4.0</v>
-      </c>
-    </row>
-    <row r="27">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>57</v>
       </c>
@@ -1549,16 +1555,16 @@
         <v>8</v>
       </c>
       <c r="D27" s="3">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E27" s="3">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F27" s="3">
-        <v>4.0</v>
-      </c>
-    </row>
-    <row r="28">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>59</v>
       </c>
@@ -1569,16 +1575,16 @@
         <v>8</v>
       </c>
       <c r="D28" s="3">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E28" s="3">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F28" s="3">
-        <v>4.0</v>
-      </c>
-    </row>
-    <row r="29">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>61</v>
       </c>
@@ -1589,16 +1595,16 @@
         <v>8</v>
       </c>
       <c r="D29" s="3">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E29" s="3">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F29" s="3">
-        <v>4.0</v>
-      </c>
-    </row>
-    <row r="30">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A30" s="4" t="s">
         <v>63</v>
       </c>
@@ -1609,16 +1615,16 @@
         <v>64</v>
       </c>
       <c r="D30" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E30" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F30" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A31" s="4" t="s">
         <v>65</v>
       </c>
@@ -1629,16 +1635,16 @@
         <v>64</v>
       </c>
       <c r="D31" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E31" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F31" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="32">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A32" s="4" t="s">
         <v>66</v>
       </c>
@@ -1649,16 +1655,16 @@
         <v>64</v>
       </c>
       <c r="D32" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E32" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F32" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A33" s="4" t="s">
         <v>13</v>
       </c>
@@ -1669,16 +1675,16 @@
         <v>64</v>
       </c>
       <c r="D33" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E33" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F33" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A34" s="4" t="s">
         <v>15</v>
       </c>
@@ -1689,16 +1695,16 @@
         <v>64</v>
       </c>
       <c r="D34" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E34" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F34" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="35">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A35" s="4" t="s">
         <v>17</v>
       </c>
@@ -1709,16 +1715,16 @@
         <v>64</v>
       </c>
       <c r="D35" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E35" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F35" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A36" s="4" t="s">
         <v>19</v>
       </c>
@@ -1729,16 +1735,16 @@
         <v>64</v>
       </c>
       <c r="D36" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E36" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F36" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A37" s="4" t="s">
         <v>21</v>
       </c>
@@ -1749,16 +1755,16 @@
         <v>64</v>
       </c>
       <c r="D37" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E37" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F37" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="38">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A38" s="4" t="s">
         <v>23</v>
       </c>
@@ -1769,16 +1775,16 @@
         <v>64</v>
       </c>
       <c r="D38" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E38" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F38" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="39">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A39" s="4" t="s">
         <v>67</v>
       </c>
@@ -1789,16 +1795,16 @@
         <v>64</v>
       </c>
       <c r="D39" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E39" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F39" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="40">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A40" s="4" t="s">
         <v>68</v>
       </c>
@@ -1809,16 +1815,16 @@
         <v>64</v>
       </c>
       <c r="D40" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E40" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F40" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="41">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A41" s="4" t="s">
         <v>70</v>
       </c>
@@ -1829,16 +1835,16 @@
         <v>64</v>
       </c>
       <c r="D41" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E41" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F41" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="42">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A42" s="4" t="s">
         <v>72</v>
       </c>
@@ -1849,16 +1855,16 @@
         <v>64</v>
       </c>
       <c r="D42" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E42" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F42" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="43">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A43" s="4" t="s">
         <v>73</v>
       </c>
@@ -1869,16 +1875,16 @@
         <v>64</v>
       </c>
       <c r="D43" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E43" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F43" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="44">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A44" s="4" t="s">
         <v>35</v>
       </c>
@@ -1889,16 +1895,16 @@
         <v>64</v>
       </c>
       <c r="D44" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E44" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F44" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="45">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A45" s="4" t="s">
         <v>37</v>
       </c>
@@ -1909,16 +1915,16 @@
         <v>64</v>
       </c>
       <c r="D45" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E45" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F45" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="46">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A46" s="4" t="s">
         <v>39</v>
       </c>
@@ -1929,16 +1935,16 @@
         <v>64</v>
       </c>
       <c r="D46" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E46" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F46" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="47">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A47" s="4" t="s">
         <v>75</v>
       </c>
@@ -1949,16 +1955,16 @@
         <v>64</v>
       </c>
       <c r="D47" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E47" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F47" s="5">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="48">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A48" s="4" t="s">
         <v>77</v>
       </c>
@@ -1969,16 +1975,16 @@
         <v>64</v>
       </c>
       <c r="D48" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E48" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F48" s="5">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="49">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A49" s="4" t="s">
         <v>79</v>
       </c>
@@ -1989,16 +1995,16 @@
         <v>64</v>
       </c>
       <c r="D49" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E49" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F49" s="5">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="50">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A50" s="4" t="s">
         <v>81</v>
       </c>
@@ -2009,16 +2015,16 @@
         <v>64</v>
       </c>
       <c r="D50" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E50" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F50" s="5">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="51">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A51" s="4" t="s">
         <v>83</v>
       </c>
@@ -2029,16 +2035,16 @@
         <v>64</v>
       </c>
       <c r="D51" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E51" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F51" s="5">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="52">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A52" s="4" t="s">
         <v>85</v>
       </c>
@@ -2049,16 +2055,16 @@
         <v>64</v>
       </c>
       <c r="D52" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E52" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F52" s="5">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="53">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A53" s="4" t="s">
         <v>87</v>
       </c>
@@ -2069,16 +2075,16 @@
         <v>64</v>
       </c>
       <c r="D53" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E53" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F53" s="5">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="54">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A54" s="4" t="s">
         <v>89</v>
       </c>
@@ -2089,16 +2095,16 @@
         <v>64</v>
       </c>
       <c r="D54" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="E54" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="F54" s="5">
-        <v>4.0</v>
-      </c>
-    </row>
-    <row r="55">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A55" s="4" t="s">
         <v>91</v>
       </c>
@@ -2109,16 +2115,16 @@
         <v>64</v>
       </c>
       <c r="D55" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E55" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F55" s="5">
-        <v>4.0</v>
-      </c>
-    </row>
-    <row r="56">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A56" s="4" t="s">
         <v>93</v>
       </c>
@@ -2129,16 +2135,16 @@
         <v>64</v>
       </c>
       <c r="D56" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E56" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F56" s="5">
-        <v>4.0</v>
-      </c>
-    </row>
-    <row r="57">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A57" s="4" t="s">
         <v>95</v>
       </c>
@@ -2149,16 +2155,16 @@
         <v>64</v>
       </c>
       <c r="D57" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E57" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F57" s="5">
-        <v>4.0</v>
-      </c>
-    </row>
-    <row r="58">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A58" s="4" t="s">
         <v>63</v>
       </c>
@@ -2169,16 +2175,16 @@
         <v>97</v>
       </c>
       <c r="D58" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E58" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F58" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="59">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A59" s="4" t="s">
         <v>98</v>
       </c>
@@ -2189,16 +2195,16 @@
         <v>97</v>
       </c>
       <c r="D59" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E59" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F59" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="60">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A60" s="4" t="s">
         <v>13</v>
       </c>
@@ -2209,16 +2215,16 @@
         <v>97</v>
       </c>
       <c r="D60" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E60" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F60" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="61">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A61" s="4" t="s">
         <v>15</v>
       </c>
@@ -2229,16 +2235,16 @@
         <v>97</v>
       </c>
       <c r="D61" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E61" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F61" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="62">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A62" s="4" t="s">
         <v>17</v>
       </c>
@@ -2249,16 +2255,16 @@
         <v>97</v>
       </c>
       <c r="D62" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E62" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F62" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="63">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A63" s="4" t="s">
         <v>19</v>
       </c>
@@ -2269,16 +2275,16 @@
         <v>97</v>
       </c>
       <c r="D63" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E63" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F63" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="64">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A64" s="4" t="s">
         <v>21</v>
       </c>
@@ -2289,16 +2295,16 @@
         <v>97</v>
       </c>
       <c r="D64" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E64" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F64" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="65">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A65" s="4" t="s">
         <v>23</v>
       </c>
@@ -2309,16 +2315,16 @@
         <v>97</v>
       </c>
       <c r="D65" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E65" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F65" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="66">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A66" s="4" t="s">
         <v>100</v>
       </c>
@@ -2329,16 +2335,16 @@
         <v>97</v>
       </c>
       <c r="D66" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E66" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F66" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="67">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A67" s="4" t="s">
         <v>102</v>
       </c>
@@ -2349,16 +2355,16 @@
         <v>97</v>
       </c>
       <c r="D67" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E67" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F67" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="68">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A68" s="4" t="s">
         <v>103</v>
       </c>
@@ -2369,16 +2375,16 @@
         <v>97</v>
       </c>
       <c r="D68" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E68" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F68" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="69">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A69" s="4" t="s">
         <v>104</v>
       </c>
@@ -2389,16 +2395,16 @@
         <v>97</v>
       </c>
       <c r="D69" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E69" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F69" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="70">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A70" s="4" t="s">
         <v>106</v>
       </c>
@@ -2409,16 +2415,16 @@
         <v>97</v>
       </c>
       <c r="D70" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E70" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F70" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="71">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A71" s="4" t="s">
         <v>35</v>
       </c>
@@ -2429,16 +2435,16 @@
         <v>97</v>
       </c>
       <c r="D71" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E71" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F71" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="72">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A72" s="4" t="s">
         <v>39</v>
       </c>
@@ -2449,16 +2455,16 @@
         <v>97</v>
       </c>
       <c r="D72" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E72" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F72" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="73">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A73" s="4" t="s">
         <v>108</v>
       </c>
@@ -2469,16 +2475,16 @@
         <v>97</v>
       </c>
       <c r="D73" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E73" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F73" s="5">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="74">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A74" s="4" t="s">
         <v>109</v>
       </c>
@@ -2489,16 +2495,16 @@
         <v>97</v>
       </c>
       <c r="D74" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E74" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F74" s="5">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="75">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A75" s="4" t="s">
         <v>110</v>
       </c>
@@ -2509,16 +2515,16 @@
         <v>97</v>
       </c>
       <c r="D75" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E75" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F75" s="5">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="76">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A76" s="4" t="s">
         <v>112</v>
       </c>
@@ -2529,16 +2535,16 @@
         <v>97</v>
       </c>
       <c r="D76" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E76" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F76" s="5">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="77">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A77" s="4" t="s">
         <v>114</v>
       </c>
@@ -2549,16 +2555,16 @@
         <v>97</v>
       </c>
       <c r="D77" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E77" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F77" s="5">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="78">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A78" s="4" t="s">
         <v>116</v>
       </c>
@@ -2569,16 +2575,16 @@
         <v>97</v>
       </c>
       <c r="D78" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E78" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F78" s="5">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="79">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A79" s="4" t="s">
         <v>118</v>
       </c>
@@ -2589,16 +2595,16 @@
         <v>97</v>
       </c>
       <c r="D79" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="E79" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="F79" s="5">
-        <v>4.0</v>
-      </c>
-    </row>
-    <row r="80">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A80" s="4" t="s">
         <v>120</v>
       </c>
@@ -2609,16 +2615,16 @@
         <v>97</v>
       </c>
       <c r="D80" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E80" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F80" s="5">
-        <v>4.0</v>
-      </c>
-    </row>
-    <row r="81">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A81" s="4" t="s">
         <v>122</v>
       </c>
@@ -2629,16 +2635,16 @@
         <v>97</v>
       </c>
       <c r="D81" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E81" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F81" s="5">
-        <v>4.0</v>
-      </c>
-    </row>
-    <row r="82">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A82" s="4" t="s">
         <v>124</v>
       </c>
@@ -2649,16 +2655,16 @@
         <v>97</v>
       </c>
       <c r="D82" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E82" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F82" s="5">
-        <v>4.0</v>
-      </c>
-    </row>
-    <row r="83">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A83" s="4" t="s">
         <v>63</v>
       </c>
@@ -2669,16 +2675,16 @@
         <v>126</v>
       </c>
       <c r="D83" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E83" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F83" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="84">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A84" s="4" t="s">
         <v>98</v>
       </c>
@@ -2689,16 +2695,16 @@
         <v>126</v>
       </c>
       <c r="D84" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E84" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F84" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="85">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A85" s="4" t="s">
         <v>13</v>
       </c>
@@ -2709,16 +2715,16 @@
         <v>126</v>
       </c>
       <c r="D85" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E85" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F85" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="86">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A86" s="4" t="s">
         <v>15</v>
       </c>
@@ -2729,16 +2735,16 @@
         <v>126</v>
       </c>
       <c r="D86" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E86" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F86" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="87">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A87" s="4" t="s">
         <v>17</v>
       </c>
@@ -2749,16 +2755,16 @@
         <v>126</v>
       </c>
       <c r="D87" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E87" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F87" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="88">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A88" s="4" t="s">
         <v>19</v>
       </c>
@@ -2769,16 +2775,16 @@
         <v>126</v>
       </c>
       <c r="D88" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E88" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F88" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="89">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A89" s="4" t="s">
         <v>21</v>
       </c>
@@ -2789,16 +2795,16 @@
         <v>126</v>
       </c>
       <c r="D89" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E89" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F89" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="90">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A90" s="4" t="s">
         <v>23</v>
       </c>
@@ -2809,16 +2815,16 @@
         <v>126</v>
       </c>
       <c r="D90" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E90" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F90" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="91">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A91" s="4" t="s">
         <v>100</v>
       </c>
@@ -2829,16 +2835,16 @@
         <v>126</v>
       </c>
       <c r="D91" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E91" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F91" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="92">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A92" s="4" t="s">
         <v>102</v>
       </c>
@@ -2849,16 +2855,16 @@
         <v>126</v>
       </c>
       <c r="D92" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E92" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F92" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="93">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A93" s="4" t="s">
         <v>103</v>
       </c>
@@ -2869,16 +2875,16 @@
         <v>126</v>
       </c>
       <c r="D93" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E93" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F93" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="94">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A94" s="4" t="s">
         <v>104</v>
       </c>
@@ -2889,16 +2895,16 @@
         <v>126</v>
       </c>
       <c r="D94" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E94" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F94" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="95">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A95" s="4" t="s">
         <v>127</v>
       </c>
@@ -2909,16 +2915,16 @@
         <v>126</v>
       </c>
       <c r="D95" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E95" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F95" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="96">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A96" s="4" t="s">
         <v>35</v>
       </c>
@@ -2929,16 +2935,16 @@
         <v>126</v>
       </c>
       <c r="D96" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E96" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F96" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="97">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A97" s="4" t="s">
         <v>39</v>
       </c>
@@ -2949,16 +2955,16 @@
         <v>126</v>
       </c>
       <c r="D97" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E97" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F97" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="98">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A98" s="4" t="s">
         <v>108</v>
       </c>
@@ -2969,16 +2975,16 @@
         <v>126</v>
       </c>
       <c r="D98" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E98" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F98" s="5">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="99">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A99" s="4" t="s">
         <v>109</v>
       </c>
@@ -2989,16 +2995,16 @@
         <v>126</v>
       </c>
       <c r="D99" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E99" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F99" s="5">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="100">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A100" s="4" t="s">
         <v>110</v>
       </c>
@@ -3009,16 +3015,16 @@
         <v>126</v>
       </c>
       <c r="D100" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E100" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F100" s="5">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="101">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A101" s="4" t="s">
         <v>129</v>
       </c>
@@ -3029,16 +3035,16 @@
         <v>126</v>
       </c>
       <c r="D101" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E101" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F101" s="5">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="102">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A102" s="4" t="s">
         <v>131</v>
       </c>
@@ -3049,16 +3055,16 @@
         <v>126</v>
       </c>
       <c r="D102" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E102" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F102" s="5">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="103">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A103" s="4" t="s">
         <v>116</v>
       </c>
@@ -3069,16 +3075,16 @@
         <v>126</v>
       </c>
       <c r="D103" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E103" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F103" s="5">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="104">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A104" s="4" t="s">
         <v>118</v>
       </c>
@@ -3089,16 +3095,16 @@
         <v>126</v>
       </c>
       <c r="D104" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="E104" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="F104" s="5">
-        <v>4.0</v>
-      </c>
-    </row>
-    <row r="105">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A105" s="4" t="s">
         <v>120</v>
       </c>
@@ -3109,16 +3115,16 @@
         <v>126</v>
       </c>
       <c r="D105" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E105" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F105" s="5">
-        <v>4.0</v>
-      </c>
-    </row>
-    <row r="106">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A106" s="4" t="s">
         <v>122</v>
       </c>
@@ -3129,16 +3135,16 @@
         <v>126</v>
       </c>
       <c r="D106" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E106" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F106" s="5">
-        <v>4.0</v>
-      </c>
-    </row>
-    <row r="107">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A107" s="4" t="s">
         <v>124</v>
       </c>
@@ -3149,32 +3155,33 @@
         <v>126</v>
       </c>
       <c r="D107" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E107" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F107" s="5">
-        <v>4.0</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:F93"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="18.63"/>
-    <col customWidth="1" min="2" max="2" width="53.88"/>
+    <col min="1" max="1" width="18.5703125" customWidth="1"/>
+    <col min="2" max="2" width="53.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3194,7 +3201,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>133</v>
       </c>
@@ -3205,16 +3212,16 @@
         <v>8</v>
       </c>
       <c r="D2" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E2" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F2" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
         <v>135</v>
       </c>
@@ -3225,16 +3232,16 @@
         <v>8</v>
       </c>
       <c r="D3" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E3" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F3" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
         <v>137</v>
       </c>
@@ -3245,16 +3252,16 @@
         <v>8</v>
       </c>
       <c r="D4" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E4" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F4" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
         <v>139</v>
       </c>
@@ -3265,16 +3272,16 @@
         <v>8</v>
       </c>
       <c r="D5" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E5" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F5" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
         <v>141</v>
       </c>
@@ -3285,16 +3292,16 @@
         <v>8</v>
       </c>
       <c r="D6" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E6" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F6" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
         <v>143</v>
       </c>
@@ -3305,16 +3312,16 @@
         <v>8</v>
       </c>
       <c r="D7" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E7" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F7" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
         <v>145</v>
       </c>
@@ -3325,16 +3332,16 @@
         <v>8</v>
       </c>
       <c r="D8" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E8" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F8" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
         <v>147</v>
       </c>
@@ -3345,16 +3352,16 @@
         <v>8</v>
       </c>
       <c r="D9" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E9" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F9" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
         <v>149</v>
       </c>
@@ -3365,16 +3372,16 @@
         <v>8</v>
       </c>
       <c r="D10" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E10" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F10" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
         <v>151</v>
       </c>
@@ -3385,16 +3392,16 @@
         <v>8</v>
       </c>
       <c r="D11" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E11" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F11" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="12">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
         <v>153</v>
       </c>
@@ -3405,16 +3412,16 @@
         <v>8</v>
       </c>
       <c r="D12" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E12" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F12" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="13">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
         <v>155</v>
       </c>
@@ -3425,16 +3432,16 @@
         <v>8</v>
       </c>
       <c r="D13" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E13" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F13" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="14">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
         <v>157</v>
       </c>
@@ -3445,16 +3452,16 @@
         <v>8</v>
       </c>
       <c r="D14" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E14" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F14" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
         <v>159</v>
       </c>
@@ -3465,16 +3472,16 @@
         <v>8</v>
       </c>
       <c r="D15" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E15" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F15" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="16">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="4" t="s">
         <v>161</v>
       </c>
@@ -3485,16 +3492,16 @@
         <v>8</v>
       </c>
       <c r="D16" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E16" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F16" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="17">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
         <v>163</v>
       </c>
@@ -3505,16 +3512,16 @@
         <v>8</v>
       </c>
       <c r="D17" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E17" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F17" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="18">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
         <v>165</v>
       </c>
@@ -3525,16 +3532,16 @@
         <v>8</v>
       </c>
       <c r="D18" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E18" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F18" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="19">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" s="4" t="s">
         <v>167</v>
       </c>
@@ -3545,16 +3552,16 @@
         <v>8</v>
       </c>
       <c r="D19" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="E19" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="F19" s="5">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="20">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" s="4" t="s">
         <v>169</v>
       </c>
@@ -3565,16 +3572,16 @@
         <v>8</v>
       </c>
       <c r="D20" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E20" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F20" s="5">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="21">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" s="4" t="s">
         <v>171</v>
       </c>
@@ -3585,16 +3592,16 @@
         <v>8</v>
       </c>
       <c r="D21" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E21" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F21" s="5">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="22">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" s="4" t="s">
         <v>173</v>
       </c>
@@ -3605,16 +3612,16 @@
         <v>8</v>
       </c>
       <c r="D22" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E22" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F22" s="5">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="23">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" s="4" t="s">
         <v>175</v>
       </c>
@@ -3625,16 +3632,16 @@
         <v>8</v>
       </c>
       <c r="D23" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E23" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F23" s="5">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="24">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A24" s="4" t="s">
         <v>177</v>
       </c>
@@ -3645,16 +3652,16 @@
         <v>8</v>
       </c>
       <c r="D24" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E24" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F24" s="5">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A25" s="4" t="s">
         <v>179</v>
       </c>
@@ -3665,16 +3672,16 @@
         <v>8</v>
       </c>
       <c r="D25" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E25" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F25" s="5">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="26">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A26" s="4" t="s">
         <v>181</v>
       </c>
@@ -3685,16 +3692,16 @@
         <v>8</v>
       </c>
       <c r="D26" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="E26" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="F26" s="5">
-        <v>4.0</v>
-      </c>
-    </row>
-    <row r="27">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A27" s="4" t="s">
         <v>183</v>
       </c>
@@ -3705,16 +3712,16 @@
         <v>64</v>
       </c>
       <c r="D27" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E27" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F27" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A28" s="4" t="s">
         <v>184</v>
       </c>
@@ -3725,16 +3732,16 @@
         <v>64</v>
       </c>
       <c r="D28" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E28" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F28" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A29" s="4" t="s">
         <v>139</v>
       </c>
@@ -3745,16 +3752,16 @@
         <v>64</v>
       </c>
       <c r="D29" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E29" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F29" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A30" s="4" t="s">
         <v>141</v>
       </c>
@@ -3765,16 +3772,16 @@
         <v>64</v>
       </c>
       <c r="D30" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E30" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F30" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A31" s="4" t="s">
         <v>143</v>
       </c>
@@ -3785,16 +3792,16 @@
         <v>64</v>
       </c>
       <c r="D31" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E31" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F31" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="32">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A32" s="4" t="s">
         <v>145</v>
       </c>
@@ -3805,16 +3812,16 @@
         <v>64</v>
       </c>
       <c r="D32" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E32" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F32" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A33" s="4" t="s">
         <v>147</v>
       </c>
@@ -3825,16 +3832,16 @@
         <v>64</v>
       </c>
       <c r="D33" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E33" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F33" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A34" s="4" t="s">
         <v>149</v>
       </c>
@@ -3845,16 +3852,16 @@
         <v>64</v>
       </c>
       <c r="D34" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E34" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F34" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="35">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A35" s="4" t="s">
         <v>185</v>
       </c>
@@ -3865,16 +3872,16 @@
         <v>64</v>
       </c>
       <c r="D35" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E35" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F35" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="36">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A36" s="4" t="s">
         <v>77</v>
       </c>
@@ -3885,16 +3892,16 @@
         <v>64</v>
       </c>
       <c r="D36" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E36" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F36" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="37">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A37" s="4" t="s">
         <v>186</v>
       </c>
@@ -3905,16 +3912,16 @@
         <v>64</v>
       </c>
       <c r="D37" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E37" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F37" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="38">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A38" s="4" t="s">
         <v>188</v>
       </c>
@@ -3925,16 +3932,16 @@
         <v>64</v>
       </c>
       <c r="D38" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E38" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F38" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="39">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A39" s="4" t="s">
         <v>159</v>
       </c>
@@ -3945,16 +3952,16 @@
         <v>64</v>
       </c>
       <c r="D39" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E39" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F39" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="40">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A40" s="4" t="s">
         <v>161</v>
       </c>
@@ -3965,16 +3972,16 @@
         <v>64</v>
       </c>
       <c r="D40" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E40" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F40" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="41">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A41" s="4" t="s">
         <v>163</v>
       </c>
@@ -3985,16 +3992,16 @@
         <v>64</v>
       </c>
       <c r="D41" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E41" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F41" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="42">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A42" s="4" t="s">
         <v>165</v>
       </c>
@@ -4005,16 +4012,16 @@
         <v>64</v>
       </c>
       <c r="D42" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E42" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F42" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="43">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A43" s="4" t="s">
         <v>189</v>
       </c>
@@ -4025,16 +4032,16 @@
         <v>64</v>
       </c>
       <c r="D43" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="E43" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="F43" s="5">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="44">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A44" s="4" t="s">
         <v>191</v>
       </c>
@@ -4045,16 +4052,16 @@
         <v>64</v>
       </c>
       <c r="D44" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E44" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F44" s="5">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="45">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A45" s="4" t="s">
         <v>193</v>
       </c>
@@ -4065,16 +4072,16 @@
         <v>64</v>
       </c>
       <c r="D45" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E45" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F45" s="5">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="46">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A46" s="4" t="s">
         <v>195</v>
       </c>
@@ -4085,16 +4092,16 @@
         <v>64</v>
       </c>
       <c r="D46" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E46" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F46" s="5">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="47">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A47" s="4" t="s">
         <v>197</v>
       </c>
@@ -4105,16 +4112,16 @@
         <v>64</v>
       </c>
       <c r="D47" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E47" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F47" s="5">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="48">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A48" s="4" t="s">
         <v>199</v>
       </c>
@@ -4125,16 +4132,16 @@
         <v>64</v>
       </c>
       <c r="D48" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E48" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F48" s="5">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="49">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A49" s="4" t="s">
         <v>201</v>
       </c>
@@ -4145,16 +4152,16 @@
         <v>64</v>
       </c>
       <c r="D49" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="E49" s="5">
-        <v>6.0</v>
+        <v>3</v>
       </c>
       <c r="F49" s="5">
-        <v>4.0</v>
-      </c>
-    </row>
-    <row r="50">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A50" s="4" t="s">
         <v>203</v>
       </c>
@@ -4165,16 +4172,16 @@
         <v>97</v>
       </c>
       <c r="D50" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E50" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F50" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="51">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A51" s="4" t="s">
         <v>204</v>
       </c>
@@ -4185,16 +4192,16 @@
         <v>97</v>
       </c>
       <c r="D51" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E51" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F51" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="52">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A52" s="4" t="s">
         <v>139</v>
       </c>
@@ -4205,16 +4212,16 @@
         <v>97</v>
       </c>
       <c r="D52" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E52" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F52" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="53">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A53" s="4" t="s">
         <v>141</v>
       </c>
@@ -4225,16 +4232,16 @@
         <v>97</v>
       </c>
       <c r="D53" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E53" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F53" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="54">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A54" s="4" t="s">
         <v>143</v>
       </c>
@@ -4245,16 +4252,16 @@
         <v>97</v>
       </c>
       <c r="D54" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E54" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F54" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="55">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A55" s="4" t="s">
         <v>145</v>
       </c>
@@ -4265,16 +4272,16 @@
         <v>97</v>
       </c>
       <c r="D55" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E55" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F55" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="56">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A56" s="4" t="s">
         <v>147</v>
       </c>
@@ -4285,16 +4292,16 @@
         <v>97</v>
       </c>
       <c r="D56" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E56" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F56" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="57">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A57" s="4" t="s">
         <v>149</v>
       </c>
@@ -4305,16 +4312,16 @@
         <v>97</v>
       </c>
       <c r="D57" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E57" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F57" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="58">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A58" s="4" t="s">
         <v>206</v>
       </c>
@@ -4325,16 +4332,16 @@
         <v>97</v>
       </c>
       <c r="D58" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E58" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F58" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="59">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A59" s="4" t="s">
         <v>208</v>
       </c>
@@ -4345,16 +4352,16 @@
         <v>97</v>
       </c>
       <c r="D59" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E59" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F59" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="60">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A60" s="4" t="s">
         <v>209</v>
       </c>
@@ -4365,16 +4372,16 @@
         <v>97</v>
       </c>
       <c r="D60" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E60" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F60" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="61">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A61" s="4" t="s">
         <v>210</v>
       </c>
@@ -4385,16 +4392,16 @@
         <v>97</v>
       </c>
       <c r="D61" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E61" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F61" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="62">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A62" s="4" t="s">
         <v>211</v>
       </c>
@@ -4405,16 +4412,16 @@
         <v>97</v>
       </c>
       <c r="D62" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E62" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F62" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="63">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A63" s="4" t="s">
         <v>159</v>
       </c>
@@ -4425,16 +4432,16 @@
         <v>97</v>
       </c>
       <c r="D63" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E63" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F63" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="64">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A64" s="4" t="s">
         <v>165</v>
       </c>
@@ -4445,16 +4452,16 @@
         <v>97</v>
       </c>
       <c r="D64" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E64" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F64" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="65">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A65" s="4" t="s">
         <v>118</v>
       </c>
@@ -4465,16 +4472,16 @@
         <v>97</v>
       </c>
       <c r="D65" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="E65" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="F65" s="5">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="66">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A66" s="4" t="s">
         <v>214</v>
       </c>
@@ -4485,16 +4492,16 @@
         <v>97</v>
       </c>
       <c r="D66" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E66" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F66" s="5">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="67">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A67" s="4" t="s">
         <v>215</v>
       </c>
@@ -4505,16 +4512,16 @@
         <v>97</v>
       </c>
       <c r="D67" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E67" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F67" s="5">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="68">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A68" s="4" t="s">
         <v>216</v>
       </c>
@@ -4525,16 +4532,16 @@
         <v>97</v>
       </c>
       <c r="D68" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E68" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F68" s="5">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="69">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A69" s="4" t="s">
         <v>218</v>
       </c>
@@ -4545,16 +4552,16 @@
         <v>97</v>
       </c>
       <c r="D69" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E69" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F69" s="5">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="70">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A70" s="4" t="s">
         <v>220</v>
       </c>
@@ -4565,16 +4572,16 @@
         <v>97</v>
       </c>
       <c r="D70" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E70" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F70" s="5">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="71">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A71" s="4" t="s">
         <v>222</v>
       </c>
@@ -4585,16 +4592,16 @@
         <v>97</v>
       </c>
       <c r="D71" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="E71" s="5">
-        <v>6.0</v>
+        <v>3</v>
       </c>
       <c r="F71" s="5">
-        <v>4.0</v>
-      </c>
-    </row>
-    <row r="72">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A72" s="4" t="s">
         <v>203</v>
       </c>
@@ -4605,16 +4612,16 @@
         <v>126</v>
       </c>
       <c r="D72" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E72" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F72" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="73">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A73" s="4" t="s">
         <v>204</v>
       </c>
@@ -4625,16 +4632,16 @@
         <v>126</v>
       </c>
       <c r="D73" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E73" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F73" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="74">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A74" s="4" t="s">
         <v>139</v>
       </c>
@@ -4645,16 +4652,16 @@
         <v>126</v>
       </c>
       <c r="D74" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E74" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F74" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="75">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A75" s="4" t="s">
         <v>141</v>
       </c>
@@ -4665,16 +4672,16 @@
         <v>126</v>
       </c>
       <c r="D75" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E75" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F75" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="76">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A76" s="4" t="s">
         <v>143</v>
       </c>
@@ -4685,16 +4692,16 @@
         <v>126</v>
       </c>
       <c r="D76" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E76" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F76" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="77">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A77" s="4" t="s">
         <v>145</v>
       </c>
@@ -4705,16 +4712,16 @@
         <v>126</v>
       </c>
       <c r="D77" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E77" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F77" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="78">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A78" s="4" t="s">
         <v>147</v>
       </c>
@@ -4725,16 +4732,16 @@
         <v>126</v>
       </c>
       <c r="D78" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E78" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F78" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="79">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A79" s="4" t="s">
         <v>149</v>
       </c>
@@ -4745,16 +4752,16 @@
         <v>126</v>
       </c>
       <c r="D79" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E79" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F79" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="80">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A80" s="4" t="s">
         <v>206</v>
       </c>
@@ -4765,16 +4772,16 @@
         <v>126</v>
       </c>
       <c r="D80" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E80" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F80" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="81">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A81" s="4" t="s">
         <v>208</v>
       </c>
@@ -4785,16 +4792,16 @@
         <v>126</v>
       </c>
       <c r="D81" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E81" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F81" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="82">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A82" s="4" t="s">
         <v>209</v>
       </c>
@@ -4805,16 +4812,16 @@
         <v>126</v>
       </c>
       <c r="D82" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E82" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F82" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="83">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A83" s="4" t="s">
         <v>210</v>
       </c>
@@ -4825,16 +4832,16 @@
         <v>126</v>
       </c>
       <c r="D83" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E83" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F83" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="84">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A84" s="4" t="s">
         <v>224</v>
       </c>
@@ -4845,16 +4852,16 @@
         <v>126</v>
       </c>
       <c r="D84" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E84" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F84" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="85">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A85" s="4" t="s">
         <v>159</v>
       </c>
@@ -4865,16 +4872,16 @@
         <v>126</v>
       </c>
       <c r="D85" s="5">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E85" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F85" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="86">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A86" s="4" t="s">
         <v>165</v>
       </c>
@@ -4885,16 +4892,16 @@
         <v>126</v>
       </c>
       <c r="D86" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E86" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="F86" s="5">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="87">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A87" s="4" t="s">
         <v>118</v>
       </c>
@@ -4905,16 +4912,16 @@
         <v>126</v>
       </c>
       <c r="D87" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="E87" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="F87" s="5">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="88">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A88" s="4" t="s">
         <v>214</v>
       </c>
@@ -4925,16 +4932,16 @@
         <v>126</v>
       </c>
       <c r="D88" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E88" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F88" s="5">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="89">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A89" s="4" t="s">
         <v>215</v>
       </c>
@@ -4945,16 +4952,16 @@
         <v>126</v>
       </c>
       <c r="D89" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E89" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F89" s="5">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="90">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A90" s="4" t="s">
         <v>226</v>
       </c>
@@ -4965,16 +4972,16 @@
         <v>126</v>
       </c>
       <c r="D90" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E90" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F90" s="5">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="91">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A91" s="4" t="s">
         <v>218</v>
       </c>
@@ -4985,16 +4992,16 @@
         <v>126</v>
       </c>
       <c r="D91" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E91" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F91" s="5">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="92">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A92" s="4" t="s">
         <v>220</v>
       </c>
@@ -5005,16 +5012,16 @@
         <v>126</v>
       </c>
       <c r="D92" s="5">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="E92" s="5">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="F92" s="5">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="93">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A93" s="4" t="s">
         <v>222</v>
       </c>
@@ -5025,33 +5032,34 @@
         <v>126</v>
       </c>
       <c r="D93" s="5">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="E93" s="5">
-        <v>6.0</v>
+        <v>3</v>
       </c>
       <c r="F93" s="5">
-        <v>4.0</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="15.88"/>
-    <col customWidth="1" min="2" max="2" width="46.88"/>
-    <col customWidth="1" min="3" max="3" width="14.88"/>
+    <col min="1" max="1" width="15.85546875" customWidth="1"/>
+    <col min="2" max="2" width="46.85546875" customWidth="1"/>
+    <col min="3" max="3" width="14.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -5071,7 +5079,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>228</v>
       </c>
@@ -5083,13 +5091,13 @@
       </c>
       <c r="D2" s="6"/>
       <c r="E2" s="7">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="F2" s="7">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>230</v>
       </c>
@@ -5100,14 +5108,14 @@
         <v>64</v>
       </c>
       <c r="D3" s="7">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E3" s="6"/>
       <c r="F3" s="7">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>232</v>
       </c>
@@ -5119,13 +5127,13 @@
       </c>
       <c r="D4" s="6"/>
       <c r="E4" s="7">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="F4" s="7">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>234</v>
       </c>
@@ -5136,14 +5144,14 @@
         <v>8</v>
       </c>
       <c r="D5" s="7">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E5" s="6"/>
       <c r="F5" s="7">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>235</v>
       </c>
@@ -5155,13 +5163,13 @@
       </c>
       <c r="D6" s="6"/>
       <c r="E6" s="7">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="F6" s="7">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>237</v>
       </c>
@@ -5172,14 +5180,14 @@
         <v>97</v>
       </c>
       <c r="D7" s="7">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E7" s="6"/>
       <c r="F7" s="7">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="8">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>235</v>
       </c>
@@ -5191,13 +5199,13 @@
       </c>
       <c r="D8" s="6"/>
       <c r="E8" s="7">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="F8" s="7">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="9">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>237</v>
       </c>
@@ -5208,14 +5216,14 @@
         <v>126</v>
       </c>
       <c r="D9" s="7">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="E9" s="6"/>
       <c r="F9" s="7">
-        <v>2.0</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>